<commit_message>
Removed much of the redundant code
</commit_message>
<xml_diff>
--- a/evaluations/classification/classification_results_LATE_FUSION_tier3_FIXED_NEW.xlsx
+++ b/evaluations/classification/classification_results_LATE_FUSION_tier3_FIXED_NEW.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T9"/>
+  <dimension ref="A1:T13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -533,14 +533,14 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>giraffes</t>
+          <t>chicks4freeid</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>1125</v>
+        <v>916</v>
       </c>
       <c r="C2" t="n">
-        <v>178</v>
+        <v>48</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
@@ -578,27 +578,27 @@
         </is>
       </c>
       <c r="M2" t="n">
-        <v>5.28</v>
+        <v>4.2</v>
       </c>
       <c r="N2" t="n">
-        <v>0.9813</v>
+        <v>0.9353</v>
       </c>
       <c r="O2" t="n">
-        <v>0.9851</v>
+        <v>0.9706</v>
       </c>
       <c r="P2" t="n">
-        <v>0.979</v>
+        <v>0.931</v>
       </c>
       <c r="Q2" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R2" t="inlineStr">
         <is>
-          <t>random</t>
+          <t>similarity-aware</t>
         </is>
       </c>
       <c r="S2" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="T2" t="inlineStr">
         <is>
@@ -654,7 +654,7 @@
         </is>
       </c>
       <c r="M3" t="n">
-        <v>9.24</v>
+        <v>5.28</v>
       </c>
       <c r="N3" t="n">
         <v>0.9813</v>
@@ -663,7 +663,7 @@
         <v>0.9851</v>
       </c>
       <c r="P3" t="n">
-        <v>0.9787</v>
+        <v>0.979</v>
       </c>
       <c r="Q3" t="b">
         <v>1</v>
@@ -685,14 +685,14 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>polarbearvidid</t>
+          <t>giraffes</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>1114</v>
+        <v>1125</v>
       </c>
       <c r="C4" t="n">
-        <v>12</v>
+        <v>178</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
@@ -730,27 +730,27 @@
         </is>
       </c>
       <c r="M4" t="n">
-        <v>1.94</v>
+        <v>9.24</v>
       </c>
       <c r="N4" t="n">
-        <v>0.8678</v>
+        <v>0.9813</v>
       </c>
       <c r="O4" t="n">
-        <v>0.9713000000000001</v>
+        <v>0.9851</v>
       </c>
       <c r="P4" t="n">
-        <v>0.8677</v>
+        <v>0.9787</v>
       </c>
       <c r="Q4" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R4" t="inlineStr">
         <is>
-          <t>similarity-aware</t>
+          <t>random</t>
         </is>
       </c>
       <c r="S4" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T4" t="inlineStr">
         <is>
@@ -761,18 +761,18 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>polarbearvidid</t>
+          <t>giraffes</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>1114</v>
+        <v>1125</v>
       </c>
       <c r="C5" t="n">
-        <v>12</v>
+        <v>178</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>ensamble</t>
+          <t>disk</t>
         </is>
       </c>
       <c r="E5" t="b">
@@ -806,27 +806,27 @@
         </is>
       </c>
       <c r="M5" t="n">
-        <v>2.14</v>
+        <v>8.19</v>
       </c>
       <c r="N5" t="n">
-        <v>0.8966</v>
+        <v>0.9739</v>
       </c>
       <c r="O5" t="n">
-        <v>0.9713000000000001</v>
+        <v>0.9776</v>
       </c>
       <c r="P5" t="n">
-        <v>0.8954</v>
+        <v>0.9718</v>
       </c>
       <c r="Q5" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R5" t="inlineStr">
         <is>
-          <t>similarity-aware</t>
+          <t>random</t>
         </is>
       </c>
       <c r="S5" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T5" t="inlineStr">
         <is>
@@ -837,14 +837,14 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>sealid</t>
+          <t>polarbearvidid</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>1663</v>
+        <v>1114</v>
       </c>
       <c r="C6" t="n">
-        <v>57</v>
+        <v>12</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
@@ -882,27 +882,27 @@
         </is>
       </c>
       <c r="M6" t="n">
-        <v>6.96</v>
+        <v>1.94</v>
       </c>
       <c r="N6" t="n">
-        <v>0.8345</v>
+        <v>0.8678</v>
       </c>
       <c r="O6" t="n">
-        <v>0.8489</v>
+        <v>0.9713000000000001</v>
       </c>
       <c r="P6" t="n">
-        <v>0.8285</v>
+        <v>0.8677</v>
       </c>
       <c r="Q6" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R6" t="inlineStr">
         <is>
-          <t>random</t>
+          <t>similarity-aware</t>
         </is>
       </c>
       <c r="S6" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="T6" t="inlineStr">
         <is>
@@ -913,14 +913,14 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>sealid</t>
+          <t>polarbearvidid</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>1663</v>
+        <v>1114</v>
       </c>
       <c r="C7" t="n">
-        <v>57</v>
+        <v>12</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
@@ -958,27 +958,27 @@
         </is>
       </c>
       <c r="M7" t="n">
-        <v>19.05</v>
+        <v>2.14</v>
       </c>
       <c r="N7" t="n">
-        <v>0.8153</v>
+        <v>0.8966</v>
       </c>
       <c r="O7" t="n">
-        <v>0.8465</v>
+        <v>0.9713000000000001</v>
       </c>
       <c r="P7" t="n">
-        <v>0.8119</v>
+        <v>0.8954</v>
       </c>
       <c r="Q7" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R7" t="inlineStr">
         <is>
-          <t>random</t>
+          <t>similarity-aware</t>
         </is>
       </c>
       <c r="S7" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="T7" t="inlineStr">
         <is>
@@ -989,18 +989,18 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>stripespotter</t>
+          <t>polarbearvidid</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>660</v>
+        <v>1114</v>
       </c>
       <c r="C8" t="n">
-        <v>46</v>
+        <v>12</v>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>ensamble</t>
+          <t>disk</t>
         </is>
       </c>
       <c r="E8" t="b">
@@ -1034,27 +1034,27 @@
         </is>
       </c>
       <c r="M8" t="n">
-        <v>2.48</v>
+        <v>1.9</v>
       </c>
       <c r="N8" t="n">
-        <v>0.9573</v>
+        <v>0.9137999999999999</v>
       </c>
       <c r="O8" t="n">
-        <v>0.9756</v>
+        <v>0.9655</v>
       </c>
       <c r="P8" t="n">
-        <v>0.9516</v>
+        <v>0.9136</v>
       </c>
       <c r="Q8" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="R8" t="inlineStr">
         <is>
-          <t>random</t>
+          <t>similarity-aware</t>
         </is>
       </c>
       <c r="S8" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="T8" t="inlineStr">
         <is>
@@ -1065,14 +1065,14 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>stripespotter</t>
+          <t>sealid</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>660</v>
+        <v>1663</v>
       </c>
       <c r="C9" t="n">
-        <v>46</v>
+        <v>57</v>
       </c>
       <c r="D9" t="inlineStr">
         <is>
@@ -1110,29 +1110,333 @@
         </is>
       </c>
       <c r="M9" t="n">
+        <v>6.96</v>
+      </c>
+      <c r="N9" t="n">
+        <v>0.8345</v>
+      </c>
+      <c r="O9" t="n">
+        <v>0.8489</v>
+      </c>
+      <c r="P9" t="n">
+        <v>0.8285</v>
+      </c>
+      <c r="Q9" t="b">
+        <v>1</v>
+      </c>
+      <c r="R9" t="inlineStr">
+        <is>
+          <t>random</t>
+        </is>
+      </c>
+      <c r="S9" t="b">
+        <v>1</v>
+      </c>
+      <c r="T9" t="inlineStr">
+        <is>
+          <t>WildlifeReID10k</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>sealid</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>1663</v>
+      </c>
+      <c r="C10" t="n">
+        <v>57</v>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>ensamble</t>
+        </is>
+      </c>
+      <c r="E10" t="b">
+        <v>1</v>
+      </c>
+      <c r="F10" t="b">
+        <v>1</v>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>megadescriptor-l-384</t>
+        </is>
+      </c>
+      <c r="H10" t="b">
+        <v>1</v>
+      </c>
+      <c r="I10" t="n">
+        <v>20</v>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>isotonic</t>
+        </is>
+      </c>
+      <c r="K10" t="n">
+        <v>200</v>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>late</t>
+        </is>
+      </c>
+      <c r="M10" t="n">
+        <v>19.05</v>
+      </c>
+      <c r="N10" t="n">
+        <v>0.8153</v>
+      </c>
+      <c r="O10" t="n">
+        <v>0.8465</v>
+      </c>
+      <c r="P10" t="n">
+        <v>0.8119</v>
+      </c>
+      <c r="Q10" t="b">
+        <v>1</v>
+      </c>
+      <c r="R10" t="inlineStr">
+        <is>
+          <t>random</t>
+        </is>
+      </c>
+      <c r="S10" t="b">
+        <v>1</v>
+      </c>
+      <c r="T10" t="inlineStr">
+        <is>
+          <t>WildlifeReID10k</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>stripespotter</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>660</v>
+      </c>
+      <c r="C11" t="n">
+        <v>46</v>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>ensamble</t>
+        </is>
+      </c>
+      <c r="E11" t="b">
+        <v>1</v>
+      </c>
+      <c r="F11" t="b">
+        <v>1</v>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>megadescriptor-l-384</t>
+        </is>
+      </c>
+      <c r="H11" t="b">
+        <v>1</v>
+      </c>
+      <c r="I11" t="n">
+        <v>20</v>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>isotonic</t>
+        </is>
+      </c>
+      <c r="K11" t="n">
+        <v>200</v>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>late</t>
+        </is>
+      </c>
+      <c r="M11" t="n">
+        <v>2.48</v>
+      </c>
+      <c r="N11" t="n">
+        <v>0.9573</v>
+      </c>
+      <c r="O11" t="n">
+        <v>0.9756</v>
+      </c>
+      <c r="P11" t="n">
+        <v>0.9516</v>
+      </c>
+      <c r="Q11" t="b">
+        <v>1</v>
+      </c>
+      <c r="R11" t="inlineStr">
+        <is>
+          <t>random</t>
+        </is>
+      </c>
+      <c r="S11" t="b">
+        <v>1</v>
+      </c>
+      <c r="T11" t="inlineStr">
+        <is>
+          <t>WildlifeReID10k</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>stripespotter</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>660</v>
+      </c>
+      <c r="C12" t="n">
+        <v>46</v>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>ensamble</t>
+        </is>
+      </c>
+      <c r="E12" t="b">
+        <v>1</v>
+      </c>
+      <c r="F12" t="b">
+        <v>1</v>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>megadescriptor-l-384</t>
+        </is>
+      </c>
+      <c r="H12" t="b">
+        <v>1</v>
+      </c>
+      <c r="I12" t="n">
+        <v>20</v>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>isotonic</t>
+        </is>
+      </c>
+      <c r="K12" t="n">
+        <v>200</v>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>late</t>
+        </is>
+      </c>
+      <c r="M12" t="n">
         <v>8.119999999999999</v>
       </c>
-      <c r="N9" t="n">
+      <c r="N12" t="n">
         <v>0.9512</v>
       </c>
-      <c r="O9" t="n">
+      <c r="O12" t="n">
         <v>0.9817</v>
       </c>
-      <c r="P9" t="n">
+      <c r="P12" t="n">
         <v>0.9509</v>
       </c>
-      <c r="Q9" t="b">
-        <v>1</v>
-      </c>
-      <c r="R9" t="inlineStr">
+      <c r="Q12" t="b">
+        <v>1</v>
+      </c>
+      <c r="R12" t="inlineStr">
         <is>
           <t>random</t>
         </is>
       </c>
-      <c r="S9" t="b">
-        <v>1</v>
-      </c>
-      <c r="T9" t="inlineStr">
+      <c r="S12" t="b">
+        <v>1</v>
+      </c>
+      <c r="T12" t="inlineStr">
+        <is>
+          <t>WildlifeReID10k</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>stripespotter</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>660</v>
+      </c>
+      <c r="C13" t="n">
+        <v>46</v>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>disk</t>
+        </is>
+      </c>
+      <c r="E13" t="b">
+        <v>1</v>
+      </c>
+      <c r="F13" t="b">
+        <v>1</v>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>megadescriptor-l-384</t>
+        </is>
+      </c>
+      <c r="H13" t="b">
+        <v>1</v>
+      </c>
+      <c r="I13" t="n">
+        <v>20</v>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>isotonic</t>
+        </is>
+      </c>
+      <c r="K13" t="n">
+        <v>200</v>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>late</t>
+        </is>
+      </c>
+      <c r="M13" t="n">
+        <v>7.62</v>
+      </c>
+      <c r="N13" t="n">
+        <v>0.9451000000000001</v>
+      </c>
+      <c r="O13" t="n">
+        <v>0.9756</v>
+      </c>
+      <c r="P13" t="n">
+        <v>0.9447</v>
+      </c>
+      <c r="Q13" t="b">
+        <v>1</v>
+      </c>
+      <c r="R13" t="inlineStr">
+        <is>
+          <t>random</t>
+        </is>
+      </c>
+      <c r="S13" t="b">
+        <v>1</v>
+      </c>
+      <c r="T13" t="inlineStr">
         <is>
           <t>WildlifeReID10k</t>
         </is>

</xml_diff>